<commit_message>
fix(consulting): harden sector classifier and regenerate RC v2
Eliminate false positives (seguro/VoIP/pavimento/saneamento metafórico/
limpeza/grama), reclassify A–C with strict evidence, fix frozen checksums
to only list staged files, and keep PENDING_HUMAN for second human review.
</commit_message>
<xml_diff>
--- a/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/pack-v2/consulting-pack.xlsx
+++ b/artifacts/campaigns/CLIENT-READY-RECURRING-CONSULTING-CYCLE-01/pack-v2/consulting-pack.xlsx
@@ -642,7 +642,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Status RC: PENDING_HUMAN | Pack: live-pack-20260725-030451-7af94c4f</t>
+          <t>Status RC: PENDING_HUMAN | Pack: live-pack-20260725-032739-85524edc</t>
         </is>
       </c>
     </row>
@@ -744,81 +744,81 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE CURITIBANOS</t>
+          <t>DEPARTAMENTO DE OBRAS E SERVIÇOS URBANOS</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>174</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MEC - UNIV. FED. DE SANTA CATARINA - SC</t>
+          <t>SECRETARIA DE INFRAESTRUTURA URBANA</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>165</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO DE OBRAS E SERVIÇOS URBANOS</t>
+          <t>PREFEITURA MUNICIPAL DE IÇARA - SC</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>149</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Secretaria de Estado da Infraestrutura …</t>
+          <t>Secretaria de Planejamento e Infraestru…</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>121</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>VIDEIRA SANEAMENTO - VISAN</t>
+          <t>MUNICÍPIO DE SÃO JOÃO DO OESTE</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>120</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL</t>
+          <t>Serviço Municipal de Água Saneamento Bá…</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>117</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE SÃO MIGUEL DO O…</t>
+          <t>Consórcio Interfederativo Santa Catarin…</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>114</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Balneário Cambo…</t>
+          <t>Secretaria de Infraestrutura</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>107</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27">
@@ -1109,12 +1109,12 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE CURITIBANOS</t>
+          <t>DEPARTAMENTO DE OBRAS E SERVIÇOS URBANOS</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>83.754.044/0001-34</t>
+          <t>82.911.249/0001-13</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -1123,29 +1123,33 @@
         </is>
       </c>
       <c r="E2" s="6" t="n">
-        <v>174</v>
+        <v>127</v>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>R$ 32.432.459,15</t>
+          <t>R$ 81.415.583,44</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>R$ 186.393,44</t>
+          <t>R$ 641.067,59</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao</t>
+          <t>drenagem, pavimentacao</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n">
@@ -1153,12 +1157,12 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>MEC - UNIV. FED. DE SANTA CATARINA - SC</t>
+          <t>SECRETARIA DE INFRAESTRUTURA URBANA</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>83.899.526/0001-82</t>
+          <t>95.815.379/0001-02</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1167,29 +1171,33 @@
         </is>
       </c>
       <c r="E3" s="6" t="n">
-        <v>165</v>
+        <v>92</v>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>R$ 998.155.532,81</t>
+          <t>R$ 13.845.577,62</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>R$ 6.049.427,47</t>
+          <t>R$ 150.495,41</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>, saneamento</t>
+          <t>drenagem, infraestrutura_urbana, pavimentacao</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="n">
@@ -1197,12 +1205,12 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO DE OBRAS E SERVIÇOS URBANOS</t>
+          <t>PREFEITURA MUNICIPAL DE IÇARA - SC</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>82.911.249/0001-13</t>
+          <t>82.916.800/0001-11</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -1211,29 +1219,33 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>149</v>
+        <v>46</v>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>R$ 93.062.512,00</t>
+          <t>R$ 29.339.085,20</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>R$ 624.580,62</t>
+          <t>R$ 637.806,20</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>, drenagem, pavimentacao</t>
+          <t>edificacoes, pavimentacao, saneamento</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
@@ -1241,12 +1253,12 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Secretaria de Estado da Infraestrutura e Mobilidade</t>
+          <t>Secretaria de Planejamento e Infraestrutura e Saneamento</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>82.951.344/0001-40</t>
+          <t>82.892.316/0001-08</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1255,29 +1267,33 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>121</v>
+        <v>76</v>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>R$ 869.613.163,67</t>
+          <t>R$ 52.230.765,58</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>R$ 7.186.885,65</t>
+          <t>R$ 687.246,92</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao, projetos</t>
+          <t>drenagem, pavimentacao</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
@@ -1285,12 +1301,12 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>VIDEIRA SANEAMENTO - VISAN</t>
+          <t>MUNICÍPIO DE SÃO JOÃO DO OESTE</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>30.753.960/0001-93</t>
+          <t>80.911.936/0001-03</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1299,29 +1315,33 @@
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>R$ 43.551.199,24</t>
+          <t>R$ 12.015.917,73</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>R$ 362.926,66</t>
+          <t>R$ 286.093,28</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>, saneamento</t>
+          <t>obras_civis, pavimentacao, saneamento</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
@@ -1329,12 +1349,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL</t>
+          <t>Serviço Municipal de Água Saneamento Básico e Infraestrutura - SEMASA</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>82.940.776/0001-56</t>
+          <t>05.472.936/0001-39</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1343,29 +1363,33 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
-        <v>117</v>
+        <v>47</v>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>R$ 3.254.020,23</t>
+          <t>R$ 34.564.663,05</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>R$ 27.812,14</t>
+          <t>R$ 735.418,36</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao</t>
+          <t>saneamento</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
@@ -1373,12 +1397,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE SÃO MIGUEL DO OESTE</t>
+          <t>Consórcio Interfederativo Santa Catarina - CINCATARINA</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>82.821.174/0001-80</t>
+          <t>12.075.748/0001-32</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1387,29 +1411,33 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>114</v>
+        <v>48</v>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>R$ 75.959.952,76</t>
+          <t>R$ 3.074.647,15</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>R$ 666.315,38</t>
+          <t>R$ 64.055,15</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>, manutencao_predial, pavimentacao, saneamento</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
@@ -1417,12 +1445,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Balneário Camboriú</t>
+          <t>Secretaria de Infraestrutura</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>83.102.285/0001-07</t>
+          <t>83.102.574/0001-06</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1431,26 +1459,26 @@
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>107</v>
+        <v>76</v>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>R$ 97.274.915,03</t>
+          <t>R$ 51.912.217,48</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>R$ 909.111,36</t>
+          <t>R$ 683.055,49</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr"/>
@@ -1461,12 +1489,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE INFRAESTRUTURA URBANA</t>
+          <t>MUNICÍPIO DE CAMPOS NOVOS</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>95.815.379/0001-02</t>
+          <t>82.939.232/0001-74</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1475,29 +1503,33 @@
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>R$ 15.104.266,50</t>
+          <t>R$ 16.254.335,20</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>R$ 151.042,67</t>
+          <t>R$ 451.509,31</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>, infraestrutura_urbana, pavimentacao</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
@@ -1505,12 +1537,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE IÇARA - SC</t>
+          <t>PREFEITURA</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>82.916.800/0001-11</t>
+          <t>82.916.826/0001-60</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1519,29 +1551,33 @@
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>94</v>
+        <v>36</v>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>R$ 59.615.325,94</t>
+          <t>R$ 15.984.818,22</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>R$ 634.205,60</t>
+          <t>R$ 444.022,73</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>, saneamento</t>
+          <t>drenagem, pavimentacao, saneamento</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
@@ -1549,12 +1585,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Secretaria de Planejamento e Infraestrutura e Saneamento</t>
+          <t>MUNICÍPIO DE PAULO LOPES</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>82.892.316/0001-08</t>
+          <t>82.892.365/0001-32</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1563,29 +1599,33 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>89</v>
+        <v>40</v>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>R$ 60.689.708,45</t>
+          <t>R$ 14.429.750,75</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>R$ 681.906,84</t>
+          <t>R$ 360.743,77</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -1593,12 +1633,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Secretaria Municipal de Planejamento - SEPLAN</t>
+          <t>Diretoria de Obras e Serviços Públicos</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>83.024.257/0001-00</t>
+          <t>82.960.758/0001-36</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1607,29 +1647,33 @@
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>R$ 208.808.752,58</t>
+          <t>R$ 25.174.569,68</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>R$ 2.456.573,56</t>
+          <t>R$ 662.488,68</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>, edificacoes</t>
+          <t>edificacoes, pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
@@ -1637,12 +1681,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE BALNEÁRIO RINCÃO</t>
+          <t>Prefeitura Municipal de Chapecó</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>17.243.084/0001-97</t>
+          <t>83.021.808/0001-82</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1651,29 +1695,33 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>85</v>
+        <v>31</v>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>R$ 50.948.099,43</t>
+          <t>R$ 75.185.575,24</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>R$ 599.389,41</t>
+          <t>R$ 2.425.341,14</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao, projetos</t>
+          <t>drenagem, edificacoes, infraestrutura_urbana, pavimentacao</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
@@ -1681,12 +1729,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>MUNICÍPIO DE SÃO JOÃO DO OESTE</t>
+          <t>PREFEITURA MUNICIPAL DE FORQUILHINHA - SC</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>80.911.936/0001-03</t>
+          <t>81.531.162/0001-58</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1695,29 +1743,33 @@
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>83</v>
+        <v>42</v>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>R$ 24.031.835,46</t>
+          <t>R$ 59.453.477,80</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>R$ 289.540,19</t>
+          <t>R$ 1.415.559,00</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao</t>
+          <t>manutencao_predial, pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
@@ -1725,12 +1777,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Consórcio Interfederativo Santa Catarina - CINCATARINA</t>
+          <t>SECRETARIA DE ADMINISTRAÇÃO E PLANEJAMENTO</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>12.075.748/0001-32</t>
+          <t>01.613.120/0001-27</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1739,29 +1791,33 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>83</v>
+        <v>27</v>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>R$ 6.006.073,99</t>
+          <t>R$ 2.779.901,25</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>R$ 72.362,34</t>
+          <t>R$ 102.959,31</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao, software</t>
+          <t>manutencao_predial, pavimentacao</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
@@ -1769,12 +1825,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Serviço Municipal de Água Saneamento Básico e Infraestrutura - SEMASA</t>
+          <t>Sombrio</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>05.472.936/0001-39</t>
+          <t>82.963.216/0001-17</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1783,29 +1839,33 @@
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>R$ 59.253.708,09</t>
+          <t>R$ 32.185.038,42</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>R$ 740.671,35</t>
+          <t>R$ 1.038.227,05</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>, saneamento</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
@@ -1813,12 +1873,12 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>SERVIÇO AUTÔNOMO MUNICIPAL DE ÁGUA E ESGOTO DE JARAGUÁ DO SUL</t>
+          <t>PREFEITURA MUNICIPAL DE ITAJAÍ - SC</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>84.438.381/0001-85</t>
+          <t>83.102.277/0001-52</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1827,29 +1887,33 @@
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>77</v>
+        <v>26</v>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>R$ 57.262.316,82</t>
+          <t>R$ 52.873.080,30</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>R$ 743.666,45</t>
+          <t>R$ 2.033.580,01</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>, saneamento</t>
+          <t>drenagem, manutencao_predial, obras_civis, pavimentacao</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J18" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
@@ -1857,12 +1921,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>SERVIÇO INTERMUNICIPAL DE ÁGUA E ESGOTO JOAÇABA HERVAL DOESTE E LUZERNA</t>
+          <t>EMASA - Empresa Municipal de Água e Saneamento de Balneário Camboriú</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>84.591.890/0001-43</t>
+          <t>07.854.402/0001-00</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1871,29 +1935,33 @@
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>77</v>
+        <v>26</v>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>R$ 17.314.313,87</t>
+          <t>R$ 43.282.724,11</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>R$ 224.861,22</t>
+          <t>R$ 1.664.720,16</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>, saneamento</t>
+          <t>saneamento</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
@@ -1901,12 +1969,12 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Secretaria de Infraestrutura</t>
+          <t>PREFEITURA MUNICIPAL DE SÃO JOÃO BATISTA</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>83.102.574/0001-06</t>
+          <t>82.925.652/0001-00</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1915,29 +1983,33 @@
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>76</v>
+        <v>37</v>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>R$ 51.912.217,48</t>
+          <t>R$ 34.732.847,77</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>R$ 683.055,49</t>
+          <t>R$ 938.725,62</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>obras_civis</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
@@ -1945,12 +2017,12 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Jaraguá do Sul</t>
+          <t>MUNICÍPIO DE TUBARÃO</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>83.102.459/0001-23</t>
+          <t>82.928.656/0001-33</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1959,29 +2031,33 @@
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>75</v>
+        <v>32</v>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>R$ 98.119.607,89</t>
+          <t>R$ 18.814.852,56</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.308.261,44</t>
+          <t>R$ 587.964,14</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>, cursos, obras_civis</t>
+          <t>manutencao_predial, pavimentacao</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n">
@@ -1989,12 +2065,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE JOAÇABA</t>
+          <t>Departamento de Planejamento, Desenvolvimento Urbanos e Indústria e Comércio</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>82.939.380/0001-99</t>
+          <t>83.102.830/0001-57</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2003,29 +2079,33 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>R$ 58.297.557,91</t>
+          <t>R$ 3.934.223,41</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>R$ 798.596,68</t>
+          <t>R$ 145.711,98</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao</t>
+          <t>pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n">
@@ -2033,12 +2113,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>SUPERINTENDENCIA REGIONAL SUL</t>
+          <t>SEOB - Secretaria de Obras de Pomerode</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>29.979.036/0001-40</t>
+          <t>83.102.251/0001-04</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2047,29 +2127,33 @@
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>R$ 43.804.496,42</t>
+          <t>R$ 21.839.288,29</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>R$ 608.395,78</t>
+          <t>R$ 753.078,91</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>manutencao_predial, saneamento</t>
+          <t>infraestrutura_urbana, pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n">
@@ -2077,12 +2161,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>MUNICÍPIO DE CAMPOS NOVOS</t>
+          <t>PREFEITURA MUNICIPAL DE MELEIRO - SC</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>82.939.232/0001-74</t>
+          <t>82.837.741/0001-96</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2091,29 +2175,33 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>R$ 32.508.670,40</t>
+          <t>R$ 6.093.831,66</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>R$ 457.868,60</t>
+          <t>R$ 304.691,58</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao</t>
+          <t>infraestrutura_urbana, obras_civis, pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n">
@@ -2121,12 +2209,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE SAO BERNARDINO</t>
+          <t>Secretário de Infraestrutura</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>01.612.812/0001-50</t>
+          <t>83.102.574/0001-06</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2135,26 +2223,26 @@
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>R$ 12.322.133,67</t>
+          <t>R$ 19.652.917,97</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>R$ 189.571,29</t>
+          <t>R$ 517.182,05</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>, cursos, obras_civis</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr"/>
@@ -2165,12 +2253,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Chapecó</t>
+          <t>PREFEITURA MUNICIPAL DE XAXIM - SC</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>83.021.808/0001-82</t>
+          <t>82.854.670/0001-30</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -2179,29 +2267,33 @@
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>62</v>
+        <v>18</v>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>R$ 140.908.025,53</t>
+          <t>R$ 17.730.435,59</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>R$ 2.272.710,09</t>
+          <t>R$ 985.024,20</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>, drenagem, edificacoes, pavimentacao</t>
+          <t>infraestrutura_urbana, pavimentacao</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J26" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n">
@@ -2209,12 +2301,12 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA</t>
+          <t>PREFEITURA MUNICIPAL DE NOVA TRENTO</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>82.916.826/0001-60</t>
+          <t>82.925.025/0001-60</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -2223,29 +2315,33 @@
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>R$ 27.402.545,52</t>
+          <t>R$ 27.535.493,77</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>R$ 441.976,54</t>
+          <t>R$ 949.499,79</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao, saneamento</t>
+          <t>obras_civis, pavimentacao</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J27" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
@@ -2253,12 +2349,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Sombrio</t>
+          <t>PREFEITURA MUNICIPAL DE TREZE DE MAIO - SC</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>82.963.216/0001-17</t>
+          <t>82.928.672/0001-26</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2267,29 +2363,33 @@
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>R$ 52.006.778,89</t>
+          <t>R$ 16.416.747,77</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>R$ 866.779,65</t>
+          <t>R$ 713.771,64</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>, drenagem, pavimentacao</t>
+          <t>manutencao_predial, obras_civis, pavimentacao</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
@@ -2297,12 +2397,12 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Diretoria de Obras e Serviços Públicos</t>
+          <t>SECRETARIA DE OBRAS E TRANSPORTES</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>82.960.758/0001-36</t>
+          <t>82.915.232/0001-34</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2311,29 +2411,33 @@
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>R$ 38.088.104,16</t>
+          <t>R$ 18.819.602,95</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>R$ 645.561,09</t>
+          <t>R$ 672.128,68</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao, terraplenagem</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
@@ -2341,12 +2445,12 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>INST.FED.DE EDUC., CIENC. E TEC. CATARINENSE</t>
+          <t>Secretaria de Administração</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>10.635.424/0001-86</t>
+          <t>83.102.228/0001-10</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2355,29 +2459,33 @@
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>R$ 102.905.638,79</t>
+          <t>R$ 10.253.157,38</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.978.954,59</t>
+          <t>R$ 394.352,21</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>, saneamento</t>
+          <t>infraestrutura_urbana, pavimentacao</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
@@ -2385,12 +2493,12 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE FORQUILHINHA - SC</t>
+          <t>MOBILIDADE URBANA</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>81.531.162/0001-58</t>
+          <t>86.051.398/0001-00</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2399,29 +2507,33 @@
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>R$ 71.402.835,48</t>
+          <t>R$ 46.132.091,18</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.373.131,45</t>
+          <t>R$ 2.096.913,24</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao, terraplenagem</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J31" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
@@ -2429,12 +2541,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE SCHROEDER - SC</t>
+          <t>PREFEITURA MUNICIPAL DE PALMITOS - SC</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>83.102.491/0001-09</t>
+          <t>85.361.863/0001-47</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -2443,29 +2555,33 @@
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>R$ 10.957.763,87</t>
+          <t>R$ 31.739.938,05</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>R$ 210.726,23</t>
+          <t>R$ 1.322.497,42</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>, saneamento, software</t>
+          <t>infraestrutura_urbana, pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J32" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
@@ -2473,12 +2589,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ADMINISTRAÇÃO E PLANEJAMENTO</t>
+          <t>MUNICÍPIO DE SANTO AMARO DA IMPERATRIZ</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>01.613.120/0001-27</t>
+          <t>82.892.324/0001-46</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2487,29 +2603,33 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>R$ 5.096.485,62</t>
+          <t>R$ 9.506.607,04</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>R$ 101.929,71</t>
+          <t>R$ 594.162,94</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>, pavimentacao, projetos</t>
+          <t>obras_civis, pavimentacao</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
@@ -2517,12 +2637,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ADMINISTRACAO</t>
+          <t>SECRETARIA MUNICIPAL DE INFRA ESTRUTURA</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>83.028.639/0001-02</t>
+          <t>82.926.569/0001-47</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2531,26 +2651,26 @@
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>R$ 11.696.716,40</t>
+          <t>R$ 12.789.758,10</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>R$ 248.866,31</t>
+          <t>R$ 412.572,84</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>, infraestrutura_urbana, obras_civis</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
       <c r="J34" s="6" t="inlineStr"/>
@@ -2561,12 +2681,12 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE ITAJAÍ - SC</t>
+          <t>Departamento de Obras Públicas</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>83.102.277/0001-52</t>
+          <t>81.140.303/0001-01</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2575,29 +2695,33 @@
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>R$ 92.114.566,14</t>
+          <t>R$ 21.063.138,66</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>R$ 2.002.490,57</t>
+          <t>R$ 957.415,39</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>, manutencao_predial, pavimentacao</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J35" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
@@ -2605,12 +2729,12 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE SÃO JOÃO BATISTA</t>
+          <t>PREFEITURA MUNICIPAL DE CORDILHEIRA ALTA - SC</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>82.925.652/0001-00</t>
+          <t>95.990.198/0001-04</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -2619,29 +2743,33 @@
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>R$ 41.851.317,33</t>
+          <t>R$ 7.153.590,03</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>R$ 909.811,25</t>
+          <t>R$ 376.504,74</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>, obras_civis, pavimentacao</t>
+          <t>obras_civis, pavimentacao, saneamento</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J36" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
@@ -2649,12 +2777,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>ADMINISTRAÇÃO</t>
+          <t>Prefeitura de Gaspar - SC</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>83.039.842/0001-84</t>
+          <t>83.102.244/0001-02</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -2663,29 +2791,33 @@
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>R$ 16.898.830,34</t>
+          <t>R$ 28.777.208,92</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>R$ 367.365,88</t>
+          <t>R$ 1.798.575,56</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>, drenagem, projetos</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J37" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
@@ -2693,12 +2825,12 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA MUNICIPAL DE AGUAS E SANEAMENTO DE LAGES - SEMASA</t>
+          <t>SECRETARIA MUNICIPAL DE OBRAS E PLANEJAMENTO</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>05.532.421/0001-87</t>
+          <t>83.102.319/0001-55</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2707,29 +2839,33 @@
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>R$ 10.694.564,03</t>
+          <t>R$ 17.884.066,11</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>R$ 232.490,52</t>
+          <t>R$ 851.622,20</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>, saneamento</t>
+          <t>drenagem, obras_civis, pavimentacao</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J38" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
@@ -2737,12 +2873,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>EMASA - Empresa Municipal de Água e Saneamento de Balneário Camboriú</t>
+          <t>MUNICÍPIO DE ORLEANS</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>07.854.402/0001-00</t>
+          <t>82.926.544/0001-43</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2751,29 +2887,33 @@
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>R$ 74.198.955,61</t>
+          <t>R$ 18.131.060,72</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.648.865,68</t>
+          <t>R$ 788.306,99</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>, saneamento</t>
+          <t>obras_civis, pavimentacao, terraplenagem</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J39" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
@@ -2781,12 +2921,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA MUNICIPAL DE OBRAS E INFRAESTRUTURA URBANA</t>
+          <t>Departamento de Urbanismo</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>82.575.812/0001-20</t>
+          <t>83.102.640/0001-30</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -2795,26 +2935,26 @@
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>R$ 32.164.002,64</t>
+          <t>R$ 18.723.510,96</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>R$ 731.000,06</t>
+          <t>R$ 668.696,82</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>, infraestrutura_urbana, pavimentacao, projetos</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
         </is>
       </c>
       <c r="J40" s="6" t="inlineStr"/>
@@ -2825,12 +2965,12 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>MUNICÍPIO DE TUBARÃO</t>
+          <t>Câmara de Vereadores de Balneário Camboriú</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>82.928.656/0001-33</t>
+          <t>83.551.549/0001-00</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -2839,29 +2979,33 @@
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>R$ 26.063.470,08</t>
+          <t>R$ 466.924,14</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>R$ 606.127,21</t>
+          <t>R$ 31.128,28</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>, manutencao_predial, pavimentacao</t>
+          <t>manutencao_predial, obras_civis</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>pncp_supplier_contracts, isolated_snapshot, engineering_filter</t>
-        </is>
-      </c>
-      <c r="J41" s="6" t="inlineStr"/>
+          <t>pncp_supplier_contracts, isolated_snapshot, engineering_reclassified</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>data_quality_score=0.85 &lt; 1.0 — ranking may over-represent entes with richer source data; not a pure market measure</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J41"/>
@@ -2963,10 +3107,14 @@
           <t>R$ 159.994.613,74</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr"/>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H2" s="6" t="inlineStr">
         <is>
-          <t>Aquisição de Rachão, Bica corrida, Material Britado, Materi… | Contratação de empresa especializada em obras e serviços de… | Contratação de empresa especializada em obras e serviços de…</t>
+          <t>Contratação de empresa especializada em obras e serviços de… | Contratação de empresa especializada em obras e serviços de… | Contratação de empresa especializada em obras e serviços de…</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
@@ -3002,7 +3150,11 @@
           <t>R$ 141.494.995,08</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Constitui objeto da presente licitação, à contratação de pe… | Constitui o objeto da presente licitação a Contratação de e… | Contratação de empresa do ramo para pavimentação asfáltica …</t>
@@ -3020,36 +3172,40 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>INFRASUL - INFRAESTUTURA E EMPREENDIMENTOS LTDA</t>
+          <t>CONSTRUTORA SCHROEDER E SCHMIDT LTDA EPP</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>03.094.645/0001-29</t>
+          <t>43.887.548/0001-08</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>concorrente_adjacente</t>
+          <t>concorrente_direto</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>R$ 177.645.328,14</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr"/>
+          <t>R$ 56.643.181,30</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Aquisição de Rachão, Bica corrida, Material Britado, Materi… | Constitui objeto da presente licitação a contratação de emp… | Constitui objeto da presente licitação, a contratação de pe…</t>
+          <t>CONCORRÊNCIA VISANDO A CONTRATAÇÃO DE EMPRESA ESPECIALIZADA… | Constitui objeto da presente licitação a Contratação de Emp… | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇ…</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=70, valor=177645328.14; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=69, valor=56643181.3; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3059,36 +3215,40 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>CONSTRUTORA SCHROEDER E SCHMIDT LTDA EPP</t>
+          <t>KAENG INFRAESTRUTURA LTDA</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>43.887.548/0001-08</t>
+          <t>22.798.043/0001-05</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>concorrente_direto</t>
+          <t>concorrente_adjacente</t>
         </is>
       </c>
       <c r="E5" s="6" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>R$ 59.936.681,30</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr"/>
+          <t>R$ 83.878.637,89</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA VISANDO A CONTRATAÇÃO DE EMPRESA ESPECIALIZADA… | Constitui objeto da presente licitação a Contratação de Emp… | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇ…</t>
+          <t>A presente licitação tem por objeto a contratação de empres… | A presente licitação tem por objeto a contratação de empres… | CONCORRÊNCIA ELETRÔNICA por EMPREITADA GLOBAL (material e m…</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=70, valor=59936681.3; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=62, valor=83878637.89; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3098,36 +3258,40 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>POLARIS SERVICOS E CONSTRUCOES LTDA-IR 1.2%</t>
+          <t>INFRASUL - INFRAESTUTURA E EMPREENDIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>12.547.887/0001-11</t>
+          <t>03.094.645/0001-29</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>concorrente_direto</t>
+          <t>concorrente_adjacente</t>
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>R$ 17.402.564,23</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr"/>
+          <t>R$ 148.114.556,25</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Contratação de serviço de manutenção do calçamento de vias …</t>
+          <t>Constitui objeto da presente licitação a contratação de emp… | Constitui objeto da presente licitação, a contratação de pe… | Constitui objeto da presente licitação, à contratação de pe…</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=70, valor=17402564.23; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=61, valor=148114556.25; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3322,11 @@
           <t>R$ 71.067.386,83</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
           <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA EM OBRAS PARA A TOTAL … | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA EM OBRAS PARA A TOTAL … | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA (EMPREITADA GLOBAL) PA…</t>
@@ -3176,12 +3344,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>FUNDACAO DE ENSINO E ENGENHARIA DE SANTA CATARINA</t>
+          <t>CCT CONSTRUTORA DE OBRAS LTDA.</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>82.895.327/0001-33</t>
+          <t>02.063.876/0001-02</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -3190,22 +3358,26 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>R$ 227.372.981,41</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr"/>
+          <t>R$ 14.796.871,13</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Apoio administrativo e financeiro para execução do Projeto …</t>
+          <t>Contratação de empresa especializada para execução (com for… | Execução (com fornecimento de mão de obra, materiais e equi…</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=59, valor=227372981.41; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=57, valor=14796871.13; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3215,36 +3387,40 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>KAENG INFRAESTRUTURA LTDA</t>
+          <t>JR CONSTRUÇÕES E TERRAPLENAGEM LTDA EPP - EPP</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>22.798.043/0001-05</t>
+          <t>05.895.635/0001-18</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>concorrente_adjacente</t>
+          <t>concorrente_direto</t>
         </is>
       </c>
       <c r="E9" s="6" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>R$ 82.520.640,58</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr"/>
+          <t>R$ 110.856.796,81</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>A presente licitação tem por objeto a contratação de empres… | A presente licitação tem por objeto a contratação de empres… | CONCORRÊNCIA ELETRÔNICA por EMPREITADA GLOBAL (material e m…</t>
+          <t>A presente licitação tem por objetivo a contratação de empr… | A presente licitação tem por objetivo a contratação de empr… | A presente licitação tem por objetivo a pavimentação asfált…</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=59, valor=82520640.58; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=56, valor=110856796.81; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3254,36 +3430,40 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>JR CONSTRUÇÕES E TERRAPLENAGEM LTDA EPP - EPP</t>
+          <t>BCL INFRAESTRUTURA LTDA.</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>05.895.635/0001-18</t>
+          <t>12.218.083/0001-79</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>concorrente_direto</t>
+          <t>concorrente_adjacente</t>
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>R$ 111.184.145,08</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr"/>
+          <t>R$ 72.385.168,83</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>A presente licitação tem por objetivo a contratação de empr… | A presente licitação tem por objetivo a contratação de empr… | A presente licitação tem por objetivo a pavimentação asfált…</t>
+          <t>A presente licitação tem por objetivo a contratação de empr… | A presente licitação tem por objeto a CONCORRÊNCIA ELETRÔNI… | Contratação de empresa de engenharia para execução de Pavim…</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=58, valor=111184145.08; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=54, valor=72385168.83; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3293,12 +3473,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>CCT CONSTRUTORA DE OBRAS LTDA.</t>
+          <t>FJ CONSTRUTORA LTDA EPP</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>02.063.876/0001-02</t>
+          <t>27.743.102/0001-53</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -3307,22 +3487,26 @@
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>R$ 14.796.871,13</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr"/>
+          <t>R$ 53.834.725,21</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para execução (com for… | Contratação eventual de serviços de reparos em redes de dre… | Contratação eventual de serviços de reparos em redes de dre…</t>
+          <t>Contratação de concreto usinado para fornecimento e aplicaç… | CONTRATAÇÃO DE EMPRESA, EM REGIME DE EMPREITADA GLOBAL, PAR… | CONTRATAÇÃO DE EMPRESA, EM REGIME DE EMPREITADA GLOBAL, PAR…</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=57, valor=14796871.13; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=51, valor=53834725.21; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3332,36 +3516,40 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>BCL INFRAESTRUTURA LTDA.</t>
+          <t>VIGA PAVIMENTAÇÃO E OBRAS LTDA</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>12.218.083/0001-79</t>
+          <t>09.223.659/0001-81</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>concorrente_adjacente</t>
+          <t>concorrente_direto</t>
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>R$ 73.227.168,83</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr"/>
+          <t>R$ 98.013.872,52</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>A presente licitação tem por objetivo a contratação de empr… | A presente licitação tem por objeto a CONCORRÊNCIA ELETRÔNI… | Contratação de empresa de engenharia para execução de Pavim…</t>
+          <t>Abertura de processo de contratação direta emergencial para… | a execução dos serviços e o fornecimento dos materiais e eq… | A presente licitação tem por objeto a contratação de empres…</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=55, valor=73227168.83; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=46, valor=98013872.52; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3371,12 +3559,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>FJ CONSTRUTORA LTDA EPP</t>
+          <t>CONSTRUTORA D. BRANGER LTDA</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>27.743.102/0001-53</t>
+          <t>34.448.864/0001-92</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -3385,22 +3573,26 @@
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>R$ 53.834.725,21</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr"/>
+          <t>R$ 41.397.367,80</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Contratação de concreto usinado para fornecimento e aplicaç… | CONTRATAÇÃO DE EMPRESA, EM REGIME DE EMPREITADA GLOBAL, PAR… | CONTRATAÇÃO DE EMPRESA, EM REGIME DE EMPREITADA GLOBAL, PAR…</t>
+          <t>Contratação de Empresa de engenharia/arquitetura para execu… | Contratação de empresa de engenharia/arquitetura para Execu… | Contratação de empresa de engenharia para execução dos serv…</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=51, valor=53834725.21; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=45, valor=41397367.8; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3410,12 +3602,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>VIGA PAVIMENTAÇÃO E OBRAS LTDA</t>
+          <t>DAVANTI ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>09.223.659/0001-81</t>
+          <t>15.129.617/0001-89</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -3424,22 +3616,26 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>R$ 116.412.862,38</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr"/>
+          <t>R$ 3.164.341,69</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>A presente licitação tem por objeto a contratação de empres… | Contratação de empresa especializada em engenharia para exe… | Contratação de empresa especializada para a execução dos se…</t>
+          <t>CONTRATAÇÃO DE EMPRESA DE ENGENHARIA ESPECIALIZADA PARA ELA… | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A ELABORAÇÃO DO P… | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA ELABORAR O PROJET…</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=46, valor=116412862.38; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=41, valor=3164341.69; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3449,12 +3645,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>CONSTRUTORA D. BRANGER LTDA</t>
+          <t>CONSTRUTORA OLIVEIRA LTDA</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>34.448.864/0001-92</t>
+          <t>80.095.466/0001-57</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -3463,22 +3659,26 @@
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>R$ 41.397.367,80</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr"/>
+          <t>R$ 115.884.123,65</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Contratação de Empresa de engenharia/arquitetura para execu… | Contratação de empresa de engenharia/arquitetura para Execu… | Contratação de empresa de engenharia para execução dos serv…</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA EM OBRAS E SERVIÇOS DE… | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A EXECUÇÃO DE OBR… | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A EXECUÇÃO DE OBR…</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=45, valor=41397367.8; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=40, valor=115884123.65; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3488,12 +3688,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>DAVANTI ENGENHARIA LTDA</t>
+          <t>CONSTRUÇÃO CIVIL MG LTDA</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>15.129.617/0001-89</t>
+          <t>06.145.928/0001-40</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -3502,22 +3702,26 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>R$ 3.164.341,69</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr"/>
+          <t>R$ 78.164.224,56</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA DE ENGENHARIA ESPECIALIZADA PARA ELA… | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A ELABORAÇÃO DO P… | CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA ELABORAR O PROJET…</t>
+          <t>A presente Licitação tem por objeto a Aquisição de materiai… | CONTRATAÇÃO DE E EMPRESA ESPECIALIZADA DE ENGENHARIA PARA A… | CONTRATAÇÃO DE E EMPRESA ESPECIALIZADA DE ENGENHARIA PARA A…</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>rank by ('n_contratos', 'valor_contratado_total'): n=41, valor=3164341.69; min_contracts&gt;=2</t>
+          <t>rank by ('n_contratos', 'valor_contratado_total'): n=37, valor=78164224.56; min_contracts&gt;=2</t>
         </is>
       </c>
     </row>
@@ -3609,22 +3813,22 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Secretaria de Estado da Infraestrutura e Mobilidade</t>
+          <t>PREFEITURA MUNICIPAL DE NAVEGANTES</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Execução dos serviços de Manutenção (Conservação/Recuperação) de Rodovias Pavimentadas e Estradas  Não  Pavimentadas  sob  a  jurisdição  da  Coordenadoria  Regional  Extremo  Oeste –SIE –CREXT (Lote  03)</t>
+          <t>CONCORRÊCIA ELETRÔNICA VISANDO A CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA FORNECIMENTO E INSTALAÇÃO DE RESERVATÓRIO METÁLICO DE 6.000 m³ NO BAIRRO SÃO DOMINGOS, PARA ATENDER AS NECESSIDADES DA SECRETARIA MUNICIPAL DE ÁGUA E SANEAMENTO BÁSICO DE NAVEGANTES/SC.</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>CEGE ENGENHARIA LTDA</t>
+          <t>CONSORCIO HABITANK NAVEGANTES</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>04.484.014/0001-89</t>
+          <t>63.077.604/0001-56</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
@@ -3634,12 +3838,12 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>R$ 60.605.734,80</t>
+          <t>R$ 10.407.000,00</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>saneamento</t>
         </is>
       </c>
       <c r="H2" s="6" t="inlineStr">
@@ -3666,22 +3870,22 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE NAVEGANTES</t>
+          <t>Unidade Única</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>CONCORRÊCIA ELETRÔNICA VISANDO A CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA FORNECIMENTO E INSTALAÇÃO DE RESERVATÓRIO METÁLICO DE 6.000 m³ NO BAIRRO SÃO DOMINGOS, PARA ATENDER AS NECESSIDADES DA SECRETARIA MUNICIPAL DE ÁGUA E SANEAMENTO BÁSICO DE NAVEGANTES/SC.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A EXECUÇÃO DOS SERVIÇOS DE CONSTRUÇÃO DE CRECHE EM TEMPO INTEGRAL PADRÃO FNDE – TIPO 01, SITUADA NA RUA LEOLÁRIO DE ARAÚJO S/Nº, BAIRRO CENTRO, ILHOTA/SC. A INTERVENÇÃO ABRANGE UMA ÁREA A CONSTRUIR DE 1.514,30M², conforme termo de referência.</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>CONSORCIO HABITANK NAVEGANTES</t>
+          <t>VB CONSTRUÇÃO CIVIL LTDA</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>63.077.604/0001-56</t>
+          <t>08.628.996/0001-96</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -3691,12 +3895,12 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>R$ 10.407.000,00</t>
+          <t>R$ 6.542.169,18</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>edificacoes</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -3723,22 +3927,22 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Unidade Única</t>
+          <t>PREFEITURA MUNICIPAL DE PALMITOS - SC</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A EXECUÇÃO DOS SERVIÇOS DE CONSTRUÇÃO DE CRECHE EM TEMPO INTEGRAL PADRÃO FNDE – TIPO 01, SITUADA NA RUA LEOLÁRIO DE ARAÚJO S/Nº, BAIRRO CENTRO, ILHOTA/SC. A INTERVENÇÃO ABRANGE UMA ÁREA A CONSTRUIR DE 1.514,30M², conforme termo de referência.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE PAVIMENTAÇÃO ASFÁLTICA E SERVIÇOS COMPLEMENTARES EM DIVERSAS RUAS DO MUNICÍPIO DE PALMITOS/SC</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>VB CONSTRUÇÃO CIVIL LTDA</t>
+          <t>GAIA RODOVIAS LTDA.</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>08.628.996/0001-96</t>
+          <t>03.257.777/0001-24</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -3748,12 +3952,12 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>R$ 6.542.169,18</t>
+          <t>R$ 1.411.572,00</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>edificacoes</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -3780,22 +3984,22 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE PALMITOS - SC</t>
+          <t>Gerência de Obras e Serviços Urbanos do Município de Massaranduba -SC</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE PAVIMENTAÇÃO ASFÁLTICA E SERVIÇOS COMPLEMENTARES EM DIVERSAS RUAS DO MUNICÍPIO DE PALMITOS/SC</t>
+          <t>PAVIMENTAÇÃO DA ESTRADA SANTO ANJO (TRECHO II) DO MUNICÍPIO DE MASSARANDUBA (SC)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>GAIA RODOVIAS LTDA.</t>
+          <t>PRO ENG CONSTRUTORA LTDA</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>03.257.777/0001-24</t>
+          <t>31.281.510/0001-08</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -3805,7 +4009,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.411.572,00</t>
+          <t>R$ 989.900,00</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -3837,22 +4041,22 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Gerência de Obras e Serviços Urbanos do Município de Massaranduba -SC</t>
+          <t>PREFEITURA MUNICIPAL DE XAXIM - SC</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>PAVIMENTAÇÃO DA ESTRADA SANTO ANJO (TRECHO II) DO MUNICÍPIO DE MASSARANDUBA (SC)</t>
+          <t>Contratação de empresa especializada, com fornecimento de materiais, mão de obra, equipamentos e insumos, para execução de obra de pavimentação asfáltica com concreto betuminoso usinado a quente (CBUQ), incluindo serviços de terraplenagem, base e sub-base, drenagem pluvial, meio-fio, sarjetas e sinalização viária na Rua Antonio Zancanaro, no Município de Xaxim-SC, conforme projeto técnico, memorial descritivo, planilha orçamentária e cronograma físico-financeiro.</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>PRO ENG CONSTRUTORA LTDA</t>
+          <t>EMBRAPAV - EMPRESA BRASILEIRA DE PAVIMENTACAO LTDA</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>31.281.510/0001-08</t>
+          <t>12.022.153/0001-19</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -3862,12 +4066,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>R$ 989.900,00</t>
+          <t>R$ 835.000,00</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>terraplenagem</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -3894,22 +4098,22 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE XAXIM - SC</t>
+          <t>Secretaria de Infraestrutura</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada, com fornecimento de materiais, mão de obra, equipamentos e insumos, para execução de obra de pavimentação asfáltica com concreto betuminoso usinado a quente (CBUQ), incluindo serviços de terraplenagem, base e sub-base, drenagem pluvial, meio-fio, sarjetas e sinalização viária na Rua Antonio Zancanaro, no Município de Xaxim-SC, conforme projeto técnico, memorial descritivo, planilha orçamentária e cronograma físico-financeiro.</t>
+          <t>Contratação de empresa especializada para execução de obras de pavimentação intertravada, drenagem pluvial e sinalização viária na Rua Palestina, Bairro Barragem, Rio do Sul/SC.</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>EMBRAPAV - EMPRESA BRASILEIRA DE PAVIMENTACAO LTDA</t>
+          <t>JC CONSTRUÇÕES E PAVIMENTAÇÕES LTDA EPP</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>12.022.153/0001-19</t>
+          <t>05.898.011/0001-54</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -3919,7 +4123,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>R$ 835.000,00</t>
+          <t>R$ 825.415,68</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -3951,22 +4155,22 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Secretaria de Infraestrutura</t>
+          <t>PREFEITURA MUNICIPAL DE ITAJAÍ - SC</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para execução de obras de pavimentação intertravada, drenagem pluvial e sinalização viária na Rua Palestina, Bairro Barragem, Rio do Sul/SC.</t>
+          <t>MÃO DE OBRA ESPECIALIZADA PARA PRESTAÇÃO DE SERVIÇOS PARA FINS DE MANUTENÇÃO PREVENTIVA E CORRETIVA DA USINA DE ASFALTO DO MUNICIPIO DE ITAJAÍ COM FORNECIMENTO DE PEÇAS ORIGINAIS/ GENUÍNAS.</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>JC CONSTRUÇÕES E PAVIMENTAÇÕES LTDA EPP</t>
+          <t>LUQUIPEÇAS LTDA ME</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>05.898.011/0001-54</t>
+          <t>09.208.545/0001-62</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -3976,7 +4180,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>R$ 825.415,68</t>
+          <t>R$ 679.999,79</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -4008,22 +4212,22 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Joinville - PMJ</t>
+          <t>MUNICÍPIO DE URUBICI</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Contratação eventual de serviços de reparos em redes de drenagem, para as Unidades Regionais de Obras.</t>
+          <t>Adesão à Ata de Registro de Preços nº 005/2024, originada do Processo Licitatório nº 018/2024 do Município de Bom Jardim da Serra/SC, cujo objeto é o Registro de Preços para contratação de empresa de engenharia para execução de serviços técnicos especializados na elaboração de projetos de pavimentação asfáltica para rodovias, ciclovias e ponte, conforme condições, especificações e exigências estabelecidas no edital e em seus anexos.</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>CCT CONSTRUTORA DE OBRAS LTDA</t>
+          <t>PROVIAS ENGENHARIA E CONSULTORIA LTDA</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>02.063.876/0001-02</t>
+          <t>23.529.844/0001-20</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -4033,12 +4237,12 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>R$ 312.473,09</t>
+          <t>R$ 103.399,98</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>drenagem</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -4065,37 +4269,37 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>MUNICÍPIO DE URUBICI</t>
+          <t>PREFEITURA MUNICIPAL DE CORDILHEIRA ALTA - SC</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Adesão à Ata de Registro de Preços nº 005/2024, originada do Processo Licitatório nº 018/2024 do Município de Bom Jardim da Serra/SC, cujo objeto é o Registro de Preços para contratação de empresa de engenharia para execução de serviços técnicos especializados na elaboração de projetos de pavimentação asfáltica para rodovias, ciclovias e ponte, conforme condições, especificações e exigências estabelecidas no edital e em seus anexos.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA REVITALIZAÇÃO DO EDIFÍCIO “MOINHO SÃO DOMINGOS”, BEM IMÓVEL TOMBADO DO MUNICÍPIO DE CORDILHEIRA ALTA/SC (DECRETO MUNICIPAL Nº 378/2022), SITUADO NA AVENIDA FERMINO TOZZO, Nº 454, BAIRRO CENTRO, CEP 89.819-000, CONFORME PROJETOS, MEMORIAL, ART E DEMAIS TERMOS DO PRESENTE EDITAL, COM VISTAS A REALIZAÇÃO DO PROJETO DENOMINADO “FÁBRICA DE CULTURA: REVITALIZAÇÃO DO MOINHO SÃO DOMINGOS”, NA FORMA DO PROCESSO Nº 2023/023189 E CONVÊNIO Nº 08/2024/FRBL, CELEBR...</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>PROVIAS ENGENHARIA E CONSULTORIA LTDA</t>
+          <t>IGM ARQUITETURA LTDA</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>23.529.844/0001-20</t>
+          <t>32.730.243/0001-71</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>R$ 103.399,98</t>
+          <t>R$ 2.660.000,00</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>infraestrutura_urbana</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -4122,37 +4326,37 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>MUNICÍPIO DE SÃO MARTINHO</t>
+          <t>MOBILIDADE URBANA</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>“Contratação de serviço de abastecimento de água tratada, coleta e tratamento de esgoto sanitário para unidades consumidoras da Prefeitura de São Martinho/SC e seus Fundos, localizados na área de concessão da Companhia Catarinense de Águas e Saneamento – CASAN, no município.”</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA FORNECIMENTO DE MATERIAIS, MÃO DE OBRA E DEMAIS OBRIGAÇÕES NECESSÁRIAS PARA EXECUÇÃO DE PAVIMENTAÇÃO EM CONCRETO DA RUA ANTÔNIO GROSSKOPF, TRECHO PARCIAL, CONTEMPLANDO OS SERVIÇOS INICIAS, DRENAGEM, PAVIMENTAÇÃO EM CONCRETO, OBRAS COMPLEMENTARES E SINALIZAÇÃO VIÁRIA, CONFORME CONDIÇÕES, QUANTIDADES E EXIGÊNCIAS ESTABELECIDAS NO TERMO DE REFERÊNCIA. O PROCESSO ESTÁ ATRELADO E CONDICIONADO A FONTE DE RECURSOS DO GOVERNO FEDERAL E CONTRAPARTIDA DA PREFEI...</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>COMPANHIA CATARINENSE DE ÁGUAS E SANEAMENTO - CASA</t>
+          <t>APA PAVIMENTACOES LTDA</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>82.508.433/0001-17</t>
+          <t>37.729.221/0001-05</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>R$ 42.428,16</t>
+          <t>R$ 1.072.000,00</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -4179,37 +4383,37 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA MUNICIPAL DE AGUAS E SANEAMENTO DE LAGES - SEMASA</t>
+          <t>Departamento de Obras Públicas</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada em Prestação de Serviços de Telefonia VoIP (Voz sobre IP), incluindo o fornecimento, a instalação, a parametrização, a migração, a portabilidade, a configuração, a ativação, o treinamento, o suporte técnico, a manutenção preventiva e corretiva, com fornecimento de peças e aparelhos para Secretaria Municipal de Águas e Saneamento (SEMASA) do Município de Lages/SC.</t>
+          <t>Contratação de empresa especializada para a execução de obras de drenagem pluvial e pavimentação asfáltica na Rua do Peixe, contemplando o Trecho I.</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>INOVA SOLUCOES EM TELECOMUNICACAO LTDA (VOXCITY)</t>
+          <t>AACS ENGENHARIA E EMPREEDIMENTOS LTDA</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>19.813.396/0001-14</t>
+          <t>15.082.833/0001-16</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>R$ 26.592,00</t>
+          <t>R$ 1.014.900,00</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -4236,37 +4440,37 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>FUNDO MUNICIPAL DE SAUDE DE SAO MARTINHO</t>
+          <t>Unidade Administrativa</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>“Contratação de serviço de abastecimento de água tratada, coleta e tratamento de esgoto sanitário para unidades consumidoras da Prefeitura de São Martinho/SC e seus Fundos, localizados na área de concessão da Companhia Catarinense de Águas e Saneamento – CASAN, no município.”</t>
+          <t>Prestação  de  serviços  de engenharia para execução de    manutenção    predial corretiva     e     preventiva, contemplando  os  serviços de   manutenção   elétrica, civil,  hidráulica  e sistema preventivo  contra  incêndio no Blaco   B   do   Centro Administrativo   da   SSP localizado   na Av.IvoSilveira,nº1521,Bloco B, BairroCapoeiras,Florianópolis-CEP:88085-000.</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>COMPANHIA CATARINENSE DE ÁGUAS E SANEAMENTO - CASA</t>
+          <t>I L AZEVEDO ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>82.508.433/0001-17</t>
+          <t>29.383.128/0001-63</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>R$ 3.346,12</t>
+          <t>R$ 416.423,27</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>obras_civis</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
@@ -4293,37 +4497,37 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>FUNDO MUNICIPAL DE ASSISTENCIA SOCIAL DE SAO MARTINHO</t>
+          <t>Unidade Administrativa</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>“Contratação de serviço de abastecimento de água tratada, coleta e tratamento de esgoto sanitário para unidades consumidoras da Prefeitura de São Martinho/SC e seus Fundos, localizados na área de concessão da Companhia Catarinense de Águas e Saneamento – CASAN, no município.”</t>
+          <t>Prestação  de  serviços  de engenharia para execução de    manutenção    predial corretiva     e     preventiva, contemplando  os  serviços de   manutenção   elétrica, civil,  hidráulica  e sistema preventivo  contra  incêndio no Blaco   B   do   Centro Administrativo   da   SSP localizado   na Av.IvoSilveira,nº1521,Bloco B, BairroCapoeiras,Florianópolis-CEP:88085-000.</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>COMPANHIA CATARINENSE DE ÁGUAS E SANEAMENTO - CASA</t>
+          <t>I L AZEVEDO ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>82.508.433/0001-17</t>
+          <t>29.383.128/0001-63</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>R$ 744,11</t>
+          <t>R$ 416.423,27</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>obras_civis</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
@@ -4350,22 +4554,22 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE CORDILHEIRA ALTA - SC</t>
+          <t>FUNDO MUNICIPAL DE SAUDE DE BELA VISTA DO TOLDO</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA REVITALIZAÇÃO DO EDIFÍCIO “MOINHO SÃO DOMINGOS”, BEM IMÓVEL TOMBADO DO MUNICÍPIO DE CORDILHEIRA ALTA/SC (DECRETO MUNICIPAL Nº 378/2022), SITUADO NA AVENIDA FERMINO TOZZO, Nº 454, BAIRRO CENTRO, CEP 89.819-000, CONFORME PROJETOS, MEMORIAL, ART E DEMAIS TERMOS DO PRESENTE EDITAL, COM VISTAS A REALIZAÇÃO DO PROJETO DENOMINADO “FÁBRICA DE CULTURA: REVITALIZAÇÃO DO MOINHO SÃO DOMINGOS”, NA FORMA DO PROCESSO Nº 2023/023189 E CONVÊNIO Nº 08/2024/FRBL, CELEBR...</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA EM OBRAS DE ENGENHARIA PARA EXECUÇÃO DA REFORMA E ADEQUAÇÃO DA COBERTURA METÁLICA DO POSTO DE SAÚDE CENTRAL DE BELA VISTA DO TOLDO/SC E DEMAIS SERVIÇOS NECESSÁRIOS.</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>IGM ARQUITETURA LTDA</t>
+          <t>HC ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>32.730.243/0001-71</t>
+          <t>48.760.149/0001-03</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -4375,12 +4579,12 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>R$ 2.660.000,00</t>
+          <t>R$ 200.802,32</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana</t>
+          <t>obras_civis</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
@@ -4407,22 +4611,22 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>MOBILIDADE URBANA</t>
+          <t>DEPARTAMENTO DE EDUCAÇÃO</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA FORNECIMENTO DE MATERIAIS, MÃO DE OBRA E DEMAIS OBRIGAÇÕES NECESSÁRIAS PARA EXECUÇÃO DE PAVIMENTAÇÃO EM CONCRETO DA RUA ANTÔNIO GROSSKOPF, TRECHO PARCIAL, CONTEMPLANDO OS SERVIÇOS INICIAS, DRENAGEM, PAVIMENTAÇÃO EM CONCRETO, OBRAS COMPLEMENTARES E SINALIZAÇÃO VIÁRIA, CONFORME CONDIÇÕES, QUANTIDADES E EXIGÊNCIAS ESTABELECIDAS NO TERMO DE REFERÊNCIA. O PROCESSO ESTÁ ATRELADO E CONDICIONADO A FONTE DE RECURSOS DO GOVERNO FEDERAL E CONTRAPARTIDA DA PREFEI...</t>
+          <t>contratação de empresa para execução das obras de construção de biblioteca e reforma de sala de aula na E.M.E.F. Frei Modesto, no município de Timbé do Sul/SC, tudo de conformidade com o projeto básico, projetos executivos, planilhas orçamentárias, memorial descritivo e demais documentos e anexos que integram este edital.</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>APA PAVIMENTACOES LTDA</t>
+          <t>CONSTRUTORA MONSANI LTDA</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>37.729.221/0001-05</t>
+          <t>14.567.961/0001-97</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
@@ -4432,17 +4636,17 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.072.000,00</t>
+          <t>R$ 194.400,00</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -4457,44 +4661,44 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Departamento de Obras Públicas</t>
+          <t>Prefeitura Municipal de Jaraguá do Sul</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para a execução de obras de drenagem pluvial e pavimentação asfáltica na Rua do Peixe, contemplando o Trecho I.</t>
+          <t>Contratação de pessoa jurídica para a prestação de serviços de engenharia, com fornecimento de materiais e mão de obra, destinados à pavimentação asfáltica, incluindo serviços preliminares, terraplenagem, drenagem pluvial, obras complementares e sinalização viária, na Rua 283 – Irmãos Maristas, no Bairro Centro, com extensão total de 969,26 m (novecentos e sessenta e nove metros e vinte e seis centímetros), em conformidade com o Anexo I – Termo de Referência, projetos, memorial descritivo, pl...</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>AACS ENGENHARIA E EMPREEDIMENTOS LTDA</t>
+          <t>PAVIPLAN PAVIMENTACAO LTDA.</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>15.082.833/0001-16</t>
+          <t>03.620.927/0001-12</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>24/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.014.900,00</t>
+          <t>R$ 919.496,94</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>terraplenagem</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -4521,37 +4725,37 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Unidade Administrativa</t>
+          <t>Serviço Autônomo Municipal de Agua e Esgoto- Blumenau SC</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Prestação  de  serviços  de engenharia para execução de    manutenção    predial corretiva     e     preventiva, contemplando  os  serviços de   manutenção   elétrica, civil,  hidráulica  e sistema preventivo  contra  incêndio no Blaco   B   do   Centro Administrativo   da   SSP localizado   na Av.IvoSilveira,nº1521,Bloco B, BairroCapoeiras,Florianópolis-CEP:88085-000.</t>
+          <t>CREDENCIAMENTO DE INSTITUIÇÕES FINANCEIRAS DEVIDAMENTE AUTORIZADAS A OPERAR PELO BANCO CENTRAL DO BRASIL, NAS MODALIDADES DE BANCO MÚLTIPLO, BANCO COMERCIAL, BANCO COOPERATIVO OU COOPERATIVA DE CRÉDITO, COM A FINALIDADE DE EXECUTAR SERVIÇOS DE ARRECADAÇÃO DE FATURAS REFERENTES AO FORNECIMENTO DE ÁGUA, ESGOTAMENTO SANITÁRIO, COLETA DE RESÍDUOS SÓLIDOS, BEM COMO DA DÍVIDA ATIVA E DEMAIS RECEITAS SOB A RESPONSABILIDADE DESTA AUTARQUIA.</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>I L AZEVEDO ENGENHARIA LTDA</t>
+          <t>BANCO COOPERATIVO SICOOB S/A</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>29.383.128/0001-63</t>
+          <t>02.038.232/0001-64</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>24/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>R$ 416.423,27</t>
+          <t>R$ 342.000,00</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>obras_civis</t>
+          <t>saneamento</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
@@ -4578,37 +4782,37 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Unidade Administrativa</t>
+          <t>Departamento de Turismo</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Prestação  de  serviços  de engenharia para execução de    manutenção    predial corretiva     e     preventiva, contemplando  os  serviços de   manutenção   elétrica, civil,  hidráulica  e sistema preventivo  contra  incêndio no Blaco   B   do   Centro Administrativo   da   SSP localizado   na Av.IvoSilveira,nº1521,Bloco B, BairroCapoeiras,Florianópolis-CEP:88085-000.</t>
+          <t>Contratação de empresa especializada no ramo da construção civil, em regime de empreitada por preço unitário, com fornecimento de materiais e mão de obra, para execução de serviços referentes a construção de edificação destinada ao quiosque na Prainha de Linha Bonita, Município de Itá/SC.</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>I L AZEVEDO ENGENHARIA LTDA</t>
+          <t>ECGT CONSTRUCOES LTDA</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>29.383.128/0001-63</t>
+          <t>06.907.152/0001-59</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>24/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>R$ 416.423,27</t>
+          <t>R$ 332.500,00</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>obras_civis</t>
+          <t>edificacoes</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
@@ -4635,37 +4839,37 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Joinville - PMJ</t>
+          <t>SECRETARIA DE ADMINISTRAÇÃO E FINANÇAS</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Contratação eventual de serviços de reparos em redes de drenagem, para as Unidades Regionais de Obras.</t>
+          <t>REF.: O PRESENTE PROCEDIMENTO LICITATÓRIO TEM POR OBJETIVO SELECIONAR A PROPOSTA MAIS VANTAJOSA PARA FUTURA E EVENTUAL A CONTRATAÇÃO DE EMPRESA DE ENGENHARIA ESPECIALIZADA PARA EXECUÇÃO DA REFORMA E REVITALIZAÇÃO DO CEMITÉRIO NA COMUNIDADE DE VILA SÃO CRISTÓVÃO, MUNICÍPIO DE SANTA ROSA DO SUL/SC, CONFORME AS ESPECIFICAÇÕES CONSTANTES NO EDITAL, CRONOGRAMA FÍSICO-FINANCEIRO, MEMORIAL DESCRITIVO, PLANILHA ORÇAMENTÁRIA, PROJETO E DEMAIS ANEXOS. (TE 0091/2026)</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>CCT CONSTRUTORA DE OBRAS LTDA</t>
+          <t>SUDOESTE CONSTRUÇÕES LTDA</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>02.063.876/0001-02</t>
+          <t>64.767.020/0001-75</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>24/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>R$ 232.343,06</t>
+          <t>R$ 200.000,00</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>drenagem</t>
+          <t>infraestrutura_urbana</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -4692,32 +4896,32 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>FUNDO MUNICIPAL DE SAUDE DE BELA VISTA DO TOLDO</t>
+          <t>Diretoria do Arquivo Público</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA EM OBRAS DE ENGENHARIA PARA EXECUÇÃO DA REFORMA E ADEQUAÇÃO DA COBERTURA METÁLICA DO POSTO DE SAÚDE CENTRAL DE BELA VISTA DO TOLDO/SC E DEMAIS SERVIÇOS NECESSÁRIOS.</t>
+          <t>Contratação  de serviços de engenharia para  execução  de manutenção predial corretiva e preventiva (via ARP 201/2025) para imóvel SIGEP 4765, sede administrativa da CODAM Criciúma, localizada na Rua José de Patta, 120, Centro, Criciúma/SC.</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>HC ENGENHARIA LTDA</t>
+          <t>AEJ ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>48.760.149/0001-03</t>
+          <t>54.960.587/0001-00</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>24/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>R$ 200.802,32</t>
+          <t>R$ 139.084,03</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -4749,42 +4953,42 @@
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO DE EDUCAÇÃO</t>
+          <t>Instituto do Meio Ambiente do Estado de Santa Catarina</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>contratação de empresa para execução das obras de construção de biblioteca e reforma de sala de aula na E.M.E.F. Frei Modesto, no município de Timbé do Sul/SC, tudo de conformidade com o projeto básico, projetos executivos, planilhas orçamentárias, memorial descritivo e demais documentos e anexos que integram este edital.</t>
+          <t>Contratação  de serviços de engenharia para  execução  de manutenção predial corretiva e preventiva (via ARP 201/2025) para imóvel SIGEP 4765, sede administrativa da CODAM Criciúma, localizada na Rua José de Patta, 120, Centro, Criciúma/SC.</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>CONSTRUTORA MONSANI LTDA</t>
+          <t>AEJ ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>14.567.961/0001-97</t>
+          <t>54.960.587/0001-00</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>24/10/2026</t>
+          <t>25/10/2026</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>R$ 194.400,00</t>
+          <t>R$ 139.084,03</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>obras_civis</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -4799,29 +5003,29 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Jaraguá do Sul</t>
+          <t>FUNDO MUNICIPAL DE SAÚDE DE BELMONTE</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Contratação de pessoa jurídica para a prestação de serviços de engenharia, com fornecimento de materiais e mão de obra, destinados à pavimentação asfáltica, incluindo serviços preliminares, terraplenagem, drenagem pluvial, obras complementares e sinalização viária, na Rua 283 – Irmãos Maristas, no Bairro Centro, com extensão total de 969,26 m (novecentos e sessenta e nove metros e vinte e seis centímetros), em conformidade com o Anexo I – Termo de Referência, projetos, memorial descritivo, pl...</t>
+          <t>CONTRATAÇÃO DE EMPRESA PARA PRESTAÇÃO DE SERVIÇOS DE MÃO DE OBRA COM FORNECIMENTO DE MATERIAIS PARA EXECUÇÃO DE OBRA DE INFRAESTRUTURA URBANA - PAVIMENTAÇÃO COM PEDRAS IRREGULARES, NO TRECHO DA RUA GENERAL OSÓRIO, COM LARGURA DE RUA DE 15,00 METROS, TOTALIZANDO ÁREA DE 845,53 M², COM LARGURA MÉDIA DE PISTA DE ROLAMENTO DE 10,00 METROS E PASSEIO LATERAL DE 2,50 METROS CADA LADO, COM RECURSOS PRÓPRIOS, DE ACORDO COM OS PROJETOS, MEMORIAL DESCRITIVO, ORÇAMENTOS, CRONOGRAMA FÍSICO FINANCEIRO E DE...</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>PAVIPLAN PAVIMENTACAO LTDA.</t>
+          <t>IMPERIAL EMPREENDIMENTOS LTDA</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>03.620.927/0001-12</t>
+          <t>02.645.439/0001-05</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -4831,7 +5035,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>R$ 919.496,94</t>
+          <t>R$ 119.000,00</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -4863,37 +5067,37 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Departamento de Turismo</t>
+          <t>PREFEITURA MUNICIPAL DE IÇARA - SC</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada no ramo da construção civil, em regime de empreitada por preço unitário, com fornecimento de materiais e mão de obra, para execução de serviços referentes a construção de edificação destinada ao quiosque na Prainha de Linha Bonita, Município de Itá/SC.</t>
+          <t>CONTRATAÇÃO DE EMPRESA OBJETIVANDO A EXECUÇÃO DA REVITALIZAÇÃO DA PRAÇA FRIDOLINO SCHUEROFF NO BAIRRO PRESIDENTE VARGAS, CONTANDO COM CERCA DE 8.605 M² DE ÁREA CONSTRUÍDA APÓS AMPLIAÇÃO.</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>ECGT CONSTRUCOES LTDA</t>
+          <t>JM PRESTADORA DE SERVIÇOS E CONSTRUÇÃO LTDA</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>06.907.152/0001-59</t>
+          <t>59.022.748/0001-38</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>25/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>R$ 332.500,00</t>
+          <t>R$ 115.672,70</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>edificacoes</t>
+          <t>infraestrutura_urbana</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
@@ -4920,42 +5124,42 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ADMINISTRAÇÃO E FINANÇAS</t>
+          <t>Secretaria Municipal de Planejamento - SEPLAN</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>REF.: O PRESENTE PROCEDIMENTO LICITATÓRIO TEM POR OBJETIVO SELECIONAR A PROPOSTA MAIS VANTAJOSA PARA FUTURA E EVENTUAL A CONTRATAÇÃO DE EMPRESA DE ENGENHARIA ESPECIALIZADA PARA EXECUÇÃO DA REFORMA E REVITALIZAÇÃO DO CEMITÉRIO NA COMUNIDADE DE VILA SÃO CRISTÓVÃO, MUNICÍPIO DE SANTA ROSA DO SUL/SC, CONFORME AS ESPECIFICAÇÕES CONSTANTES NO EDITAL, CRONOGRAMA FÍSICO-FINANCEIRO, MEMORIAL DESCRITIVO, PLANILHA ORÇAMENTÁRIA, PROJETO E DEMAIS ANEXOS. (TE 0091/2026)</t>
+          <t>Serviços de manutenção predial preventiva, corretiva, bem como reformas prediais sem acréscimo de área construída, abrangendo as áreas civil, elétrica, hidráulica e de sistemas preventivos de combate a incêndio, em todas as unidades administrativas sob responsabilidade do Município de Concórdia.</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>SUDOESTE CONSTRUÇÕES LTDA</t>
+          <t>CONSTRUTORA FOSCARINI EIRELI</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>64.767.020/0001-75</t>
+          <t>11.517.944/0001-57</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>25/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>R$ 200.000,00</t>
+          <t>R$ 3.880.000,00</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana</t>
+          <t>manutencao_predial</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -4970,44 +5174,44 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Diretoria do Arquivo Público</t>
+          <t>PREFEITURA MUNICIPAL DE ITAJAÍ - SC</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Contratação  de serviços de engenharia para  execução  de manutenção predial corretiva e preventiva (via ARP 201/2025) para imóvel SIGEP 4765, sede administrativa da CODAM Criciúma, localizada na Rua José de Patta, 120, Centro, Criciúma/SC.</t>
+          <t>CONTRATAÇÃO DE EMPRESA PARA EXECUÇÃO DAS OBRAS DE PAVIMENTAÇÃO, DRENAGEM PLUVIAL, PASSEIO PÚBLICO E SINALIZAÇÃO VERTICAL NA RUA AUGUSTO CUGNIER</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>AEJ ENGENHARIA LTDA</t>
+          <t>C R ARTEFATOS DE CIMENTO LTDA</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>54.960.587/0001-00</t>
+          <t>01.650.178/0001-40</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>25/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>R$ 139.084,03</t>
+          <t>R$ 3.269.997,63</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>obras_civis</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
@@ -5034,37 +5238,37 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Instituto do Meio Ambiente do Estado de Santa Catarina</t>
+          <t>Serviços Urbanos</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Contratação  de serviços de engenharia para  execução  de manutenção predial corretiva e preventiva (via ARP 201/2025) para imóvel SIGEP 4765, sede administrativa da CODAM Criciúma, localizada na Rua José de Patta, 120, Centro, Criciúma/SC.</t>
+          <t>Contratação de empresa especializada para a execução de pavimentação em concreto rígido, drenagem pluvial e sinalização viária da Rua Prefeito August Heinrich Purnhagen, localizada no Bairro Universitário, Taió/SC, com extensão de 865,00 metros</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>AEJ ENGENHARIA LTDA</t>
+          <t>MILENIUM SOLUCOES E SERVICOS LTDA</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>54.960.587/0001-00</t>
+          <t>05.594.191/0001-80</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>25/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>R$ 139.084,03</t>
+          <t>R$ 1.885.100,00</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>obras_civis</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
@@ -5091,37 +5295,37 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>FUNDO MUNICIPAL DE SAÚDE DE BELMONTE</t>
+          <t>DIRETORIA DE TURISMO</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA PARA PRESTAÇÃO DE SERVIÇOS DE MÃO DE OBRA COM FORNECIMENTO DE MATERIAIS PARA EXECUÇÃO DE OBRA DE INFRAESTRUTURA URBANA - PAVIMENTAÇÃO COM PEDRAS IRREGULARES, NO TRECHO DA RUA GENERAL OSÓRIO, COM LARGURA DE RUA DE 15,00 METROS, TOTALIZANDO ÁREA DE 845,53 M², COM LARGURA MÉDIA DE PISTA DE ROLAMENTO DE 10,00 METROS E PASSEIO LATERAL DE 2,50 METROS CADA LADO, COM RECURSOS PRÓPRIOS, DE ACORDO COM OS PROJETOS, MEMORIAL DESCRITIVO, ORÇAMENTOS, CRONOGRAMA FÍSICO FINANCEIRO E DE...</t>
+          <t>CONTRATAÇÃO DE PESSOA JURÍDICA PARA PRESTAÇÃO DE SERVIÇOS DE ENGENHARIA COM FORNECIMENTO DE MATERIAIS, EQUIPAMENTOS E MÃO DE OBRA PARA CONSTRUÇÃO DE PORTAL DE ENTRADA E REVITALIZAÇÃO DA RUA TRENTO, BAIRRO DIVINÉIA, NO MUNICÍPIO DE RIO DOS CEDROS/SC, EM CONFORMIDADE COM O PROJETO BÁSICO, MEMORIAL DESCRITIVO E DEMAIS ANEXOS DO EDITAL.</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>IMPERIAL EMPREENDIMENTOS LTDA</t>
+          <t>F9 CONSTRUTORA LTDA</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>02.645.439/0001-05</t>
+          <t>50.032.977/0001-69</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>25/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>R$ 119.000,00</t>
+          <t>R$ 753.000,00</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>infraestrutura_urbana</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
@@ -5148,37 +5352,37 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Blumenau</t>
+          <t>TRIBUNAL REGIONAL DO TRABALHO DA 12A.REGIAO</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Contratação de Empresa Especializada em prestação de serviços gerais de limpeza e conservação, jardinagem e roçadas, limpeza e manutenção de pátios, áreas pavimentadas e áreas gramadas, compreendendo o fornecimento de mão de obra, uniformes e equipamentos adequados à execução dos serviços, no Parque Ramiro Ruediger , Parque Alcântaro Corrêa, Ginásio de Esportes Sebastião Cruz e Parque Vila Germânica. Conforme especificações constantes neste edital e anexos. SECTUR.</t>
+          <t>Adequação e reforma do 7º pavimento do prédio sede para instalação de 2 (dois) gabinetes de desembargadores.</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>AJ CANE CONSTRUÇÕES LTDA</t>
+          <t>LAMINA CONSTRUCOES LTDA</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>40.680.039/0001-11</t>
+          <t>19.534.597/0001-82</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.359.000,00</t>
+          <t>R$ 350.987,50</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>reformas</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
@@ -5205,32 +5409,32 @@
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE IÇARA - SC</t>
+          <t>Prefeitura Municipal de Chapecó</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA OBJETIVANDO A EXECUÇÃO DA REVITALIZAÇÃO DA PRAÇA FRIDOLINO SCHUEROFF NO BAIRRO PRESIDENTE VARGAS, CONTANDO COM CERCA DE 8.605 M² DE ÁREA CONSTRUÍDA APÓS AMPLIAÇÃO.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE REVITALIZAÇÃO DA ILUMINAÇÃO DA PONTE ENTRE A DIVISA DE SANTA CATARINA (CHAPECÓ) COM O RIO GRANDE DO SUL (NONOAI).</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>JM PRESTADORA DE SERVIÇOS E CONSTRUÇÃO LTDA</t>
+          <t>ELETROTEC SISTEMAS DE ENERGIA LTDA</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>59.022.748/0001-38</t>
+          <t>11.796.575/0001-89</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>R$ 115.672,70</t>
+          <t>R$ 318.000,00</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
@@ -5262,42 +5466,42 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Serviço Autônomo Municipal de Agua e Esgoto- Blumenau SC</t>
+          <t>SECRETARIA MUNICIPAL DE PLANEJAMENTO E DESENVOLVIMENTO ECONÔMICO SUSTENTÁVEL</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa para prestação de seguro de veículos pertencentes à frota do Serviço Autônomo Municipal de Água e Esgoto de Blumenau/SC.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A ELABORAÇÃO DE PROJETO DE ENGENHARIA EM NÍVEL EXECUTIVO VISANDO A EXTENSÃO DE VIA ATÉ A PONTE SOBRE O RIO PIÇARRAS, BEM COMO PARA A REALIZAÇÃO DE ESTUDOS, PROGRAMAS, PLANOS E PROJETOS AMBIENTAIS, INCLUINDO COMPLEMENTAÇÕES E ACOMPANHAMENTO DOS PROCESSOS DE LICENCIAMENTO AMBIENTAL.</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>GENTE SEGURADORA SA</t>
+          <t>GEOMAPA ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>90.180.605/0001-02</t>
+          <t>03.339.646/0001-96</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>27/10/2026</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>R$ 54.555,00</t>
+          <t>R$ 163.980,00</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -5312,29 +5516,29 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Joinville - PMJ</t>
+          <t>MUNICÍPIO DE URUBICI</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para preparação da base, fornecimento e instalação de campo de grama sintética, padrão FIFA Quality Pro, sistema de drenagem e sistema de irrigação do Estádio Arena Joinville.</t>
+          <t>Contratação de empresa especializada para elaboração de projetos técnicos necessários à reforma do salão do CTG – CENTRO DE TRADIÇOES GAÚCHAS - URUBICI contemplando: Projeto Preventivo contra Incêndio (PPCI), projeto hidrossanitário, projeto elétrico, projeto de gás, projeto de climatização, projeto estrutural (área de expansão), com todo acervo necessário, de acordo com o projeto arquitetônico em anexo.</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Playpiso Pisos Esportivos Ltda</t>
+          <t>ALTITUDE ENGENHARIA LTDA</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>57.396.418/0001-87</t>
+          <t>42.792.909/0001-70</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
@@ -5344,17 +5548,17 @@
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>R$ 4.008.000,00</t>
+          <t>R$ 27.000,00</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>drenagem</t>
+          <t>projetos</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -5369,49 +5573,49 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_HIGH_CONFIDENCE</t>
+          <t>ENGINEERING_REVIEW</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Secretaria Municipal de Planejamento - SEPLAN</t>
+          <t>SECRETARIA DE INFRAESTRUTURA URBANA</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Serviços de manutenção predial preventiva, corretiva, bem como reformas prediais sem acréscimo de área construída, abrangendo as áreas civil, elétrica, hidráulica e de sistemas preventivos de combate a incêndio, em todas as unidades administrativas sob responsabilidade do Município de Concórdia.</t>
+          <t>Contratação de empresa especializada para prestação de serviços de pavimentação de vias urbanas, localizadas junto ao Bairro São Miguel, localizadas nesta cidade de Fraiburgo/SC, conforme especificações deste Termo, Projetos, Memoriais Descritivos e Quantitativos (anexos ao PAL e parte dele integrante):</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>CONSTRUTORA FOSCARINI EIRELI</t>
+          <t>RA PAVIMENTAÇÕES LTDA</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>11.517.944/0001-57</t>
+          <t>33.062.208/0001-94</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>R$ 3.880.000,00</t>
+          <t>R$ 2.626.200,00</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>manutencao_predial</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -5426,39 +5630,39 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>PREFEITURA MUNICIPAL DE ITAJAÍ - SC</t>
+          <t>Secretaria de Educação, Esporte e Cultura</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA PARA EXECUÇÃO DAS OBRAS DE PAVIMENTAÇÃO, DRENAGEM PLUVIAL, PASSEIO PÚBLICO E SINALIZAÇÃO VERTICAL NA RUA AUGUSTO CUGNIER</t>
+          <t>CONCORRÊNCIA ELETRÔNICA PARA CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA REALIZAR ASFALTAMENTO DAS RUAS PADRE ADALBERTO ORTHMANN, PADRE FRANZ E ALWIN WEINRICH, LOCALIZADAS NO CENTRO DO MUNICÍPIO DE PRESIDENTE GETÚLIO.</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>C R ARTEFATOS DE CIMENTO LTDA</t>
+          <t>FJ CONSTRUTORA LTDA</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>01.650.178/0001-40</t>
+          <t>27.743.102/0001-53</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>R$ 3.269.997,63</t>
+          <t>R$ 1.050.000,00</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
@@ -5490,32 +5694,32 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Serviços Urbanos</t>
+          <t>SECRETARIA DE INFRAESTRUTURA URBANA</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para a execução de pavimentação em concreto rígido, drenagem pluvial e sinalização viária da Rua Prefeito August Heinrich Purnhagen, localizada no Bairro Universitário, Taió/SC, com extensão de 865,00 metros</t>
+          <t>Pavimentação em pedras irregulares de basalto nas Ruas "A" Trecho II, "B" Trecho III e "H" no Bairro Nossa Senhora Aparecida.</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>MILENIUM SOLUCOES E SERVICOS LTDA</t>
+          <t>J.M.A TERRAPLANAGEM LTDA</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>05.594.191/0001-80</t>
+          <t>43.637.217/0001-10</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>R$ 1.885.100,00</t>
+          <t>R$ 589.998,72</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -5547,37 +5751,37 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>DIRETORIA DE TURISMO</t>
+          <t>Fundação Municipal de Esportes - Fme</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE PESSOA JURÍDICA PARA PRESTAÇÃO DE SERVIÇOS DE ENGENHARIA COM FORNECIMENTO DE MATERIAIS, EQUIPAMENTOS E MÃO DE OBRA PARA CONSTRUÇÃO DE PORTAL DE ENTRADA E REVITALIZAÇÃO DA RUA TRENTO, BAIRRO DIVINÉIA, NO MUNICÍPIO DE RIO DOS CEDROS/SC, EM CONFORMIDADE COM O PROJETO BÁSICO, MEMORIAL DESCRITIVO E DEMAIS ANEXOS DO EDITAL.</t>
+          <t>Execução de serviços de engenharia para Manutenção Predial e Civil das edificações do município de Indaial e de seus fundos e fundações.</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>F9 CONSTRUTORA LTDA</t>
+          <t>CONSTRUTORA SCHROEDER E SCHMIDT LTDA</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>50.032.977/0001-69</t>
+          <t>43.887.548/0001-08</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>R$ 753.000,00</t>
+          <t>R$ 134.268,71</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana</t>
+          <t>obras_civis</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
@@ -5604,37 +5808,37 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>TRIBUNAL REGIONAL DO TRABALHO DA 12A.REGIAO</t>
+          <t>Prefeitura Municipal de Trombudo Central - SC</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Adequação e reforma do 7º pavimento do prédio sede para instalação de 2 (dois) gabinetes de desembargadores.</t>
+          <t>AQUISIÇÃO DE EQUIPAMENTO DE PINTURA E DEMARCAÇÃO VIÁRIA DO TIPO AIRLESS,  DESTINADO À APLICAÇÃO DE TINTA EM SINALIZAÇÃO HORIZONTAL, CONTEMPLANDO PINTURA DE MEIO-FIO, EIXO DE CENTRO (1 OU 2 FAIXAS), FAIXAS DE PEDESTRES E LOMBADAS, COM CAPACIDADE OPERACIONAL E ESPECIFICAÇÕES TÉCNICAS ADEQUADAS PARA ATENDER AOS PADRÕES DE SEGURANÇA VIÁRIA ESTABELECIDOS PELA LEGISLAÇÃO VIGENTE. O EQUIPAMENTO SERÁ UTILIZADO PELAS EQUIPES MUNICIPAIS NA EXECUÇÃO E MANUTENÇÃO DA SINALIZAÇÃO VIÁRIA DE RUAS E VIAS PÚBL...</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>LAMINA CONSTRUCOES LTDA</t>
+          <t>SD COMERCIAL EQUIPAMENTOS LTDA</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>19.534.597/0001-82</t>
+          <t>44.802.526/0001-60</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>R$ 350.987,50</t>
+          <t>R$ 34.000,00</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>pavimentacao</t>
+          <t>drenagem</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
@@ -5661,37 +5865,37 @@
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>Prefeitura Municipal de Chapecó</t>
+          <t>Prefeitura Municipal de Catanduvas</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE REVITALIZAÇÃO DA ILUMINAÇÃO DA PONTE ENTRE A DIVISA DE SANTA CATARINA (CHAPECÓ) COM O RIO GRANDE DO SUL (NONOAI).</t>
+          <t>Contratação de empresa especializada para execução de pavimentação nos estacionamentos centrais do Município, com fornecimento de matérias e mão de obra, conforme descritos no projeto, memorial descritivo e termo de referência (Anexo “II”) do presente edital.</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>ELETROTEC SISTEMAS DE ENERGIA LTDA</t>
+          <t>R3 PRESTACAO DE SERVICOS LTDA</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>11.796.575/0001-89</t>
+          <t>15.371.451/0001-02</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>R$ 318.000,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>infraestrutura_urbana</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
@@ -5718,42 +5922,42 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>SECRETARIA MUNICIPAL DE PLANEJAMENTO E DESENVOLVIMENTO ECONÔMICO SUSTENTÁVEL</t>
+          <t>EMASA - Empresa Municipal de Água e Saneamento de Balneário Camboriú</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A ELABORAÇÃO DE PROJETO DE ENGENHARIA EM NÍVEL EXECUTIVO VISANDO A EXTENSÃO DE VIA ATÉ A PONTE SOBRE O RIO PIÇARRAS, BEM COMO PARA A REALIZAÇÃO DE ESTUDOS, PROGRAMAS, PLANOS E PROJETOS AMBIENTAIS, INCLUINDO COMPLEMENTAÇÕES E ACOMPANHAMENTO DOS PROCESSOS DE LICENCIAMENTO AMBIENTAL.</t>
+          <t>AQUISIÇÃO DE CONJUNTOS MOTOBOMBAS SUBMERSÍVEIS PARA SEREM UTILIZADOS NO SISTEMA DE ESGOTAMENTO SANITÁRIO, NO MUNICÍPIO DE BALNEÁRIO CAMBORIÚ/SC.</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>GEOMAPA ENGENHARIA LTDA</t>
+          <t>SULZER PUMPS WASTEWATER BRASIL LTDA</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>03.339.646/0001-96</t>
+          <t>77.153.260/0013-65</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>R$ 163.980,00</t>
+          <t>R$ 6.454.000,00</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>saneamento</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -5768,44 +5972,44 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>FUNDO MUNICIPAL DE EDUCAÇÃO</t>
+          <t>Secretaria Municipal de Planejamento</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Dispensa de licitação para contratação de assessoria técnica especializada em infraestrutura educacional para saneamento de inconformidades e tramitação de processos de prestação de contas das obras, celebrados entre o município de Porto Belo (SC) e o Fundo Nacional de Desenvolvimento da Educação (FNDE).</t>
+          <t>Contratação de empresa para execução de projeto de construção da obra de pavimentação asfáltica e drenagem da Estrada Geral Fazenda de Dentro (Rua Manoel Mendes), Localidade de Fazenda de Dentro,Biguaçu/SC</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>MC PROJETOS E ASSESSORIA LTDA</t>
+          <t>CONSTRUCOES SCHOROEDER LTDA</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>31.302.767/0001-07</t>
+          <t>10.249.046/0001-00</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>R$ 27.000,00</t>
+          <t>R$ 1.325.157,30</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
@@ -5832,42 +6036,42 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>MUNICÍPIO DE URUBICI</t>
+          <t>PREFEITURA MUNICIPAL DE BELA VISTA DO TOLDO - SC</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para elaboração de projetos técnicos necessários à reforma do salão do CTG – CENTRO DE TRADIÇOES GAÚCHAS - URUBICI contemplando: Projeto Preventivo contra Incêndio (PPCI), projeto hidrossanitário, projeto elétrico, projeto de gás, projeto de climatização, projeto estrutural (área de expansão), com todo acervo necessário, de acordo com o projeto arquitetônico em anexo.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA EXECUÇÃO DE RECUPERAÇÃO DE PAVIMENTAÇÃO ASFÁLTICA NA RUA AUGUSTO KUCHLER.</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>ALTITUDE ENGENHARIA LTDA</t>
+          <t>EPG ENGENHARIA E CONSTRUCOES LTDA</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>42.792.909/0001-70</t>
+          <t>34.605.142/0001-02</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>27/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>R$ 27.000,00</t>
+          <t>R$ 598.403,21</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>projetos</t>
+          <t>pavimentacao</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -5882,7 +6086,7 @@
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>ENGINEERING_REVIEW</t>
+          <t>ENGINEERING_HIGH_CONFIDENCE</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6791,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>live-pack-20260725-030451-7af94c4f</t>
+          <t>live-pack-20260725-032739-85524edc</t>
         </is>
       </c>
     </row>
@@ -6611,7 +6815,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>c17864f681776e7d12df1bd99edb7f4c8f89f4c4</t>
+          <t>7706783a722d7b0a1469aa73b2d2a402b10117ae</t>
         </is>
       </c>
     </row>
@@ -6695,7 +6899,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>{'eligible_population': 1179237, 'active_contracts': 1179237, 'uf_filter': 'SC', 'period_min': '2023-07-20', 'period_max': '2026-07-23', 'sample_label': 'FULL_ELIGIBLE_POPULATION', 'not_sample_of_n': True, 'n_orgaos_eligible': 820, 'n_contracts_eligible': 14177, 'n_contracts_eligible_engineering': 14177, 'valor_sum_eligible': 9693935892.64, 'export_limit': 40, 'export_is_not_universe': True, 'ranking_metric': 'engineering_activity_not_general_volume', 'profile_object_terms': ['paviment', 'drenagem', 'terrapl', 'saneamento', 'reforma predial', 'manutencao predial', 'construcao de edif', 'ampliacao de', 'obra de engenharia', 'infraestrutura urbana', 'projeto', 'construcao de edificio', 'construcao de predio', 'edificacao publica', 'predio publico', 'pavimentacao', 'pavimentacao asfaltica', 'capeamento asfaltico', 'drenagem urbana', 'galeria pluvial']}</t>
+          <t>{'eligible_population': 1179237, 'active_contracts': 1179237, 'uf_filter': 'SC', 'period_min': '2023-07-20', 'period_max': '2026-07-23', 'sample_label': 'FULL_ELIGIBLE_POPULATION', 'not_sample_of_n': True, 'n_orgaos_eligible': 801, 'n_contracts_eligible': 13604, 'n_contracts_eligible_engineering': 13604, 'valor_sum_eligible': 8639092667.5, 'export_limit': 40, 'export_is_not_universe': True, 'ranking_metric': 'engineering_activity_not_general_volume', 'ranking_method': 'SQL prefilter by engineering terms + per-organ sample reclassification via sector_classifier; qtd/valor adjusted by engineering sample ratio', 'profile_object_terms': ['pavimentacao', 'drenagem urbana', 'terrapl', 'saneamento basico', 'reforma predial', 'manutencao predial', 'construcao de edif', 'ampliacao de', 'obra de engenharia', 'infraestrutura urbana', 'projeto', 'construcao de edificio', 'construcao de predio', 'edificacao publica', 'predio publico', 'pavimentacao asfaltica', 'capeamento asfaltico', 'drenagem', 'galeria pluvial', 'sarjeta']}</t>
         </is>
       </c>
     </row>

</xml_diff>